<commit_message>
Open with the introduction, as the framework orders it
The game now runs Start -> Rules -> the Hook -> Map (framework 3.1-3.2).
Start is the introduction: it says this is a mystery game for practicing
HEAR and shows the four HEAR moves; the Rules follow, then the Hook.
New game text: start.intro, start.hear_title, start.hear_note, start.next,
rules.next, hook.next.

Packet: headings and labels now use the framework's terms (the CCC,
the Hook, Situation, Assignment, Position on the CCC, Clues, Red Herrings,
Response Matrix).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/engine/HEARsay game text.xlsx
+++ b/engine/HEARsay game text.xlsx
@@ -566,12 +566,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Title screen: series name, title, the scenario's summary and the map.</t>
+          <t>Introduction, part 1: the game and a brief summary of HEAR (the hear.* text), with the title, the scenario's summary and the map.</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>The scenario's hook text comes from the Response Matrix (Passages sheet, 'the Hook').</t>
+          <t>Shown after the introduction, then the Map. The scenario's Hook text comes from the Response Matrix (Passages sheet, 'the Hook').</t>
         </is>
       </c>
     </row>
@@ -615,7 +615,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Shown once after the Hook.</t>
+          <t>Introduction, part 2: the rules. Shown once after Start; then the Hook.</t>
         </is>
       </c>
     </row>
@@ -890,7 +890,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F121"/>
+  <dimension ref="A1:F124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1412,7 +1412,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>start.begin</t>
+          <t>start.intro</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1422,13 +1422,17 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Begin</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr"/>
+          <t>This is a mystery game, and a chance to practice the HEAR framework as you play. You solve the case by interviewing witnesses, and how receptively you talk to them decides how much they tell you.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>paraphrase</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr"/>
@@ -1436,17 +1440,17 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>hook.assignment</t>
+          <t>start.hear_title</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Hook</t>
+          <t>Start</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Your assignment</t>
+          <t>The HEAR framework</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
@@ -1460,23 +1464,27 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>hook.mystery</t>
+          <t>start.hear_note</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Hook</t>
+          <t>Start</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>The mystery</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr"/>
+          <t>The HEAR guide stays in the sidebar, so you can come back to it at any time.</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>paraphrase</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr"/>
@@ -1484,17 +1492,17 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>hook.ccc</t>
+          <t>start.next</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Hook</t>
+          <t>Start</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>What the campus is fighting about: {ccc}</t>
+          <t>How to play</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
@@ -1508,7 +1516,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>hook.read_rules</t>
+          <t>hook.assignment</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1518,7 +1526,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Read the rules</t>
+          <t>Your assignment</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr"/>
@@ -1532,17 +1540,17 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>rules.title</t>
+          <t>hook.mystery</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Rules</t>
+          <t>Hook</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>How to play</t>
+          <t>The mystery</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
@@ -1556,27 +1564,23 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>rules.1</t>
+          <t>hook.ccc</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Rules</t>
+          <t>Hook</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>There are {n_witnesses} witnesses. You can visit them in any order and go back to them, and ask each of them any of the same {n_questions} questions.</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>3.1</t>
-        </is>
-      </c>
+          <t>What the campus is fighting about: {ccc}</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>paraphrase</t>
+          <t>label</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr"/>
@@ -1584,27 +1588,23 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>rules.2</t>
+          <t>hook.next</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Rules</t>
+          <t>Hook</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>You have {budget} questions in total, across all witnesses. That is not enough to ask everything, so choose. Re-reading an answer you already have is free.</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>3.1</t>
-        </is>
-      </c>
+          <t>Go to the campus map</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>paraphrase</t>
+          <t>label</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr"/>
@@ -1612,7 +1612,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>rules.3</t>
+          <t>rules.title</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1622,17 +1622,13 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>For each witness, one question is a tripwire: it offends them and they walk away for good. The tripwire costs a question. Read each witness's background card for hints about what they would resent.</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>3.1</t>
-        </is>
-      </c>
+          <t>How to play</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>paraphrase</t>
+          <t>label</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr"/>
@@ -1640,7 +1636,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>rules.4</t>
+          <t>rules.1</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1650,12 +1646,12 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Every answer gives you a piece of information and the witness's opinion about {ccc}. Some information is useful, some is a red herring that a careful reasoner can rule out.</t>
+          <t>There are {n_witnesses} witnesses. You can visit them in any order and go back to them, and ask each of them any of the same {n_questions} questions.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1668,7 +1664,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>rules.5</t>
+          <t>rules.2</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1678,7 +1674,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Pay attention to how each witness expresses their opinion. Some do it receptively, using HEAR; some do not. At the end you will rank the witnesses from most to least receptive, for bonus points.</t>
+          <t>You have {budget} questions in total, across all witnesses. That is not enough to ask everything, so choose. Re-reading an answer you already have is free.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1696,7 +1692,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>rules.6</t>
+          <t>rules.3</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1706,12 +1702,12 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Once per witness, after any answer, you may ask a follow-up about their opinion. You pick between two phrasings. The receptive phrasing earns the next Major Clue and the next letter of H-E-A-R. The other one ends the interview. Follow-ups do not cost a question.</t>
+          <t>For each witness, one question is a tripwire: it offends them and they walk away for good. The tripwire costs a question. Read each witness's background card for hints about what they would resent.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>3.3.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1724,7 +1720,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>rules.7</t>
+          <t>rules.4</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1734,12 +1730,12 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>There are {n_major} Major Clues. Together they make the solution clear. A successful follow-up after all of them are earned gives bonus points.</t>
+          <t>Every answer gives you a piece of information and the witness's opinion about {ccc}. Some information is useful, some is a red herring that a careful reasoner can rule out.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>3.3.1</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1752,7 +1748,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>rules.8</t>
+          <t>rules.5</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1762,12 +1758,12 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>You can solve the case at any time, but only once. When your questions run out, you must submit.</t>
+          <t>Pay attention to how each witness expresses their opinion. Some do it receptively, using HEAR; some do not. At the end you will rank the witnesses from most to least receptive, for bonus points.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1780,7 +1776,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>rules.9</t>
+          <t>rules.6</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1790,12 +1786,12 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>The Evidence board keeps everything you have learned. The HEAR guide and these rules are always in the sidebar.</t>
+          <t>Once per witness, after any answer, you may ask a follow-up about their opinion. You pick between two phrasings. The receptive phrasing earns the next Major Clue and the next letter of H-E-A-R. The other one ends the interview. Follow-ups do not cost a question.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>3.3.1</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -1808,7 +1804,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>rules.go_to_map</t>
+          <t>rules.7</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1818,13 +1814,17 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Go to the campus map</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr"/>
+          <t>There are {n_major} Major Clues. Together they make the solution clear. A successful follow-up after all of them are earned gives bonus points.</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>3.3.1</t>
+        </is>
+      </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>paraphrase</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr"/>
@@ -1832,22 +1832,22 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>hear.title</t>
+          <t>rules.8</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>HEAR Guide</t>
+          <t>Rules</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>The HEAR framework</t>
+          <t>You can solve the case at any time, but only once. When your questions run out, you must submit.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -1860,22 +1860,22 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>hear.intro</t>
+          <t>rules.9</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>HEAR Guide</t>
+          <t>Rules</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Conversational receptiveness is a willingness to engage with opposing views, shown through the words you use. Research by Julia Minson and colleagues found four markers that make someone come across as receptive:</t>
+          <t>The Evidence board keeps everything you have learned. The HEAR guide and these rules are always in the sidebar.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -1888,27 +1888,23 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>hear.H.move</t>
+          <t>rules.next</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>HEAR Guide</t>
+          <t>Rules</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Hedge your claims</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>Begin the case</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr"/>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>verbatim</t>
+          <t>label</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr"/>
@@ -1916,7 +1912,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>hear.H.text</t>
+          <t>hear.title</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -1926,7 +1922,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Signal that you might be wrong: “I think”, “it's possible that”, “I could be misreading this”.</t>
+          <t>The HEAR framework</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -1944,7 +1940,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>hear.E.move</t>
+          <t>hear.intro</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -1954,7 +1950,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Emphasize agreement</t>
+          <t>Conversational receptiveness is a willingness to engage with opposing views, shown through the words you use. Research by Julia Minson and colleagues found four markers that make someone come across as receptive:</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1964,7 +1960,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>verbatim</t>
+          <t>paraphrase</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr"/>
@@ -1972,7 +1968,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>hear.E.text</t>
+          <t>hear.H.move</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -1982,7 +1978,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Name the common ground, even partial: “We both want…”, “I agree that…”.</t>
+          <t>Hedge your claims</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1992,7 +1988,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>paraphrase</t>
+          <t>verbatim</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr"/>
@@ -2000,7 +1996,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>hear.A.move</t>
+          <t>hear.H.text</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2010,7 +2006,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Acknowledge the other's perspective</t>
+          <t>Signal that you might be wrong: “I think”, “it's possible that”, “I could be misreading this”.</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -2020,7 +2016,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>verbatim</t>
+          <t>paraphrase</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr"/>
@@ -2028,7 +2024,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>hear.A.text</t>
+          <t>hear.E.move</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2038,7 +2034,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Show you have understood the other view, accurately and fairly: “I understand that you…”, “You're right that…”.</t>
+          <t>Emphasize agreement</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2048,7 +2044,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>paraphrase</t>
+          <t>verbatim</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr"/>
@@ -2056,7 +2052,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>hear.R.move</t>
+          <t>hear.E.text</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2066,7 +2062,7 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Reframe to the positive</t>
+          <t>Name the common ground, even partial: “We both want…”, “I agree that…”.</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -2076,7 +2072,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>verbatim</t>
+          <t>paraphrase</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr"/>
@@ -2084,7 +2080,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>hear.R.text</t>
+          <t>hear.A.move</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -2094,7 +2090,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Say what you want rather than what you oppose, and avoid contradictions and dismissals such as “that's wrong” or “no one serious thinks…”.</t>
+          <t>Acknowledge the other's perspective</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2104,7 +2100,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>paraphrase</t>
+          <t>verbatim</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr"/>
@@ -2112,7 +2108,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>hear.unreceptive</t>
+          <t>hear.A.text</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -2122,12 +2118,12 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Unreceptive language states opinions flatly, generalizes about the other person, attributes motives, or dismisses them. Listen for both kinds as the witnesses talk about the controversy.</t>
+          <t>Show you have understood the other view, accurately and fairly: “I understand that you…”, “You're right that…”.</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -2140,23 +2136,27 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>case.title</t>
+          <t>hear.R.move</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Case File</t>
+          <t>HEAR Guide</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Case file</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr"/>
+          <t>Reframe to the positive</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>verbatim</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr"/>
@@ -2164,23 +2164,27 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>case.mystery</t>
+          <t>hear.R.text</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Case File</t>
+          <t>HEAR Guide</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>The mystery</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr"/>
+          <t>Say what you want rather than what you oppose, and avoid contradictions and dismissals such as “that's wrong” or “no one serious thinks…”.</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>paraphrase</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr"/>
@@ -2188,23 +2192,27 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>case.brief</t>
+          <t>hear.unreceptive</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Case File</t>
+          <t>HEAR Guide</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Your brief</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr"/>
+          <t>Unreceptive language states opinions flatly, generalizes about the other person, attributes motives, or dismisses them. Listen for both kinds as the witnesses talk about the controversy.</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>paraphrase</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr"/>
@@ -2212,7 +2220,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>case.ccc</t>
+          <t>case.title</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -2222,7 +2230,7 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>The controversy: {ccc}</t>
+          <t>Case file</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr"/>
@@ -2236,17 +2244,17 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>map.title</t>
+          <t>case.mystery</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Map</t>
+          <t>Case File</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Campus map</t>
+          <t>The mystery</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr"/>
@@ -2260,17 +2268,17 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>map.note</t>
+          <t>case.brief</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Map</t>
+          <t>Case File</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Choose a witness to interview. Their background card is shown before you ask anything.</t>
+          <t>Your brief</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr"/>
@@ -2284,17 +2292,17 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>map.asked</t>
+          <t>case.ccc</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Map</t>
+          <t>Case File</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>{n} asked</t>
+          <t>The controversy: {ccc}</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr"/>
@@ -2303,16 +2311,12 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
+      <c r="F54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>map.not_yet</t>
+          <t>map.title</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -2322,7 +2326,7 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Not yet interviewed</t>
+          <t>Campus map</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr"/>
@@ -2336,7 +2340,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>map.walked_away</t>
+          <t>map.note</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -2346,7 +2350,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Walked away</t>
+          <t>Choose a witness to interview. Their background card is shown before you ask anything.</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr"/>
@@ -2360,7 +2364,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>map.follow_up_used</t>
+          <t>map.asked</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -2370,7 +2374,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>· follow-up used</t>
+          <t>{n} asked</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr"/>
@@ -2379,22 +2383,26 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>interview.found_at</t>
+          <t>map.not_yet</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Interview</t>
+          <t>Map</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Found at: {location}</t>
+          <t>Not yet interviewed</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr"/>
@@ -2403,26 +2411,22 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>location</t>
-        </is>
-      </c>
+      <c r="F58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>interview.closed</t>
+          <t>map.walked_away</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Interview</t>
+          <t>Map</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>{name} has walked away and will not answer any more questions.</t>
+          <t>Walked away</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr"/>
@@ -2431,26 +2435,22 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
+      <c r="F59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>interview.reread</t>
+          <t>map.follow_up_used</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Interview</t>
+          <t>Map</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Re-read: {question}</t>
+          <t>· follow-up used</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr"/>
@@ -2459,26 +2459,22 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
-        <is>
-          <t>question</t>
-        </is>
-      </c>
+      <c r="F60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>answer.you_asked</t>
+          <t>interview.found_at</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Answer</t>
+          <t>Interview</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>You asked {name}:</t>
+          <t>Found at: {location}</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr"/>
@@ -2489,34 +2485,30 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>location</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>answer.tripwire</t>
+          <t>interview.closed</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Answer</t>
+          <t>Interview</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>That was {name}'s tripwire. The interview is over.</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>3.1</t>
-        </is>
-      </c>
+          <t>{name} has walked away and will not answer any more questions.</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr"/>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>paraphrase</t>
+          <t>label</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -2528,17 +2520,17 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>answer.ask_else</t>
+          <t>interview.reread</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Answer</t>
+          <t>Interview</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Ask {first_name} something else</t>
+          <t>Re-read: {question}</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr"/>
@@ -2549,24 +2541,24 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>first_name</t>
+          <t>question</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>followup.title</t>
+          <t>answer.you_asked</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>Answer</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Follow-up with {name}</t>
+          <t>You asked {name}:</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr"/>
@@ -2584,22 +2576,22 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>followup.note</t>
+          <t>answer.tripwire</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>Answer</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Choose how to press {first_name} about their view. You get one follow-up per witness, and it does not cost a question. Choose carefully: one phrasing will open them up, the other will end the interview.</t>
+          <t>That was {name}'s tripwire. The interview is over.</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>3.3.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -2609,24 +2601,24 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>first_name</t>
+          <t>name</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>followup.not_now</t>
+          <t>answer.ask_else</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>Answer</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Not now</t>
+          <t>Ask {first_name} something else</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr"/>
@@ -2635,22 +2627,26 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>first_name</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>result_fu.opens_up</t>
+          <t>followup.title</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Follow-up Result</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>{name} opens up</t>
+          <t>Follow-up with {name}</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr"/>
@@ -2668,67 +2664,63 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>result_fu.major</t>
+          <t>followup.note</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Follow-up Result</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Major Clue {n}: {mc_title}</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr"/>
+          <t>Choose how to press {first_name} about their view. You get one follow-up per witness, and it does not cost a question. Choose carefully: one phrasing will open them up, the other will end the interview.</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>3.3.1</t>
+        </is>
+      </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>paraphrase</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>n mc_title</t>
+          <t>first_name</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>result_fu.all_earned</t>
+          <t>followup.not_now</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Follow-up Result</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>You already hold every Major Clue, so {name} has nothing new to add, but the question lands well. Bonus: +{bonus}.</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>3.3.1</t>
-        </is>
-      </c>
+          <t>Not now</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr"/>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>paraphrase</t>
-        </is>
-      </c>
-      <c r="F69" s="2" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>result_fu.why</t>
+          <t>result_fu.opens_up</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -2738,7 +2730,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Why that phrasing worked</t>
+          <t>{name} opens up</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr"/>
@@ -2747,12 +2739,16 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F70" s="2" t="inlineStr"/>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>result_fu.walks_away</t>
+          <t>result_fu.major</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -2762,7 +2758,7 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>{name} walks away</t>
+          <t>Major Clue {n}: {mc_title}</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr"/>
@@ -2773,14 +2769,14 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>n mc_title</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>result_fu.not_receptive</t>
+          <t>result_fu.all_earned</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -2790,7 +2786,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>That follow-up was not receptive. {name}'s interview is over.</t>
+          <t>You already hold every Major Clue, so {name} has nothing new to add, but the question lands well. Bonus: +{bonus}.</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -2812,7 +2808,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>result_fu.continue</t>
+          <t>result_fu.why</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -2822,7 +2818,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Continue the interview</t>
+          <t>Why that phrasing worked</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr"/>
@@ -2836,17 +2832,17 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>evidence.title</t>
+          <t>result_fu.walks_away</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Evidence Board</t>
+          <t>Follow-up Result</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Evidence board</t>
+          <t>{name} walks away</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr"/>
@@ -2855,46 +2851,58 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F74" s="2" t="inlineStr"/>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>evidence.major</t>
+          <t>result_fu.not_receptive</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Evidence Board</t>
+          <t>Follow-up Result</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Major Clues</t>
-        </is>
-      </c>
-      <c r="D75" s="2" t="inlineStr"/>
+          <t>That follow-up was not receptive. {name}'s interview is over.</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>3.3.1</t>
+        </is>
+      </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>label</t>
-        </is>
-      </c>
-      <c r="F75" s="2" t="inlineStr"/>
+          <t>paraphrase</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>evidence.major_none</t>
+          <t>result_fu.continue</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Evidence Board</t>
+          <t>Follow-up Result</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>None yet. Earn them with receptive follow-up questions.</t>
+          <t>Continue the interview</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr"/>
@@ -2908,7 +2916,7 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>evidence.notes</t>
+          <t>evidence.title</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -2918,7 +2926,7 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Notes (in the order you heard them)</t>
+          <t>Evidence board</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr"/>
@@ -2932,7 +2940,7 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>evidence.notes_none</t>
+          <t>evidence.major</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -2942,7 +2950,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Nothing yet.</t>
+          <t>Major Clues</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr"/>
@@ -2956,7 +2964,7 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>evidence.source</t>
+          <t>evidence.major_none</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -2966,7 +2974,7 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>— {name}, asked “{question}”</t>
+          <t>None yet. Earn them with receptive follow-up questions.</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr"/>
@@ -2975,16 +2983,12 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F79" s="2" t="inlineStr">
-        <is>
-          <t>name question</t>
-        </is>
-      </c>
+      <c r="F79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>evidence.witnesses</t>
+          <t>evidence.notes</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -2994,7 +2998,7 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Witnesses</t>
+          <t>Notes (in the order you heard them)</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr"/>
@@ -3008,7 +3012,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>evidence.n_asked</t>
+          <t>evidence.notes_none</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -3018,7 +3022,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>{n} question(s) asked</t>
+          <t>Nothing yet.</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr"/>
@@ -3027,16 +3031,12 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F81" s="2" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
+      <c r="F81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>evidence.walked_tripwire</t>
+          <t>evidence.source</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -3046,7 +3046,7 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>walked away (tripwire)</t>
+          <t>— {name}, asked “{question}”</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr"/>
@@ -3055,12 +3055,16 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F82" s="2" t="inlineStr"/>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>name question</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>evidence.walked_followup</t>
+          <t>evidence.witnesses</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -3070,7 +3074,7 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>walked away (follow-up)</t>
+          <t>Witnesses</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr"/>
@@ -3084,7 +3088,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>evidence.good_followup</t>
+          <t>evidence.n_asked</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -3094,7 +3098,7 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>receptive follow-up</t>
+          <t>{n} question(s) asked</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr"/>
@@ -3103,12 +3107,16 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>evidence.bonus</t>
+          <t>evidence.walked_tripwire</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -3118,7 +3126,7 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Bonus points so far: {points}</t>
+          <t>walked away (tripwire)</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr"/>
@@ -3127,26 +3135,22 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F85" s="2" t="inlineStr">
-        <is>
-          <t>points</t>
-        </is>
-      </c>
+      <c r="F85" s="2" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>submit.title</t>
+          <t>evidence.walked_followup</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Submission</t>
+          <t>Evidence Board</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Solve the case</t>
+          <t>walked away (follow-up)</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr"/>
@@ -3160,27 +3164,23 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>submit.once</t>
+          <t>evidence.good_followup</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Submission</t>
+          <t>Evidence Board</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>You can submit only once. Check your Evidence board first.</t>
-        </is>
-      </c>
-      <c r="D87" s="2" t="inlineStr">
-        <is>
-          <t>3.4</t>
-        </is>
-      </c>
+          <t>receptive follow-up</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr"/>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>paraphrase</t>
+          <t>label</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr"/>
@@ -3188,17 +3188,17 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>submit.choose</t>
+          <t>evidence.bonus</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Submission</t>
+          <t>Evidence Board</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>— choose —</t>
+          <t>Bonus points so far: {points}</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr"/>
@@ -3207,12 +3207,16 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F88" s="2" t="inlineStr"/>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>points</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>submit.both</t>
+          <t>submit.title</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -3222,7 +3226,7 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Choose an answer for both questions.</t>
+          <t>Solve the case</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr"/>
@@ -3236,7 +3240,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>submit.submit</t>
+          <t>submit.once</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -3246,13 +3250,17 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Submit my solution</t>
-        </is>
-      </c>
-      <c r="D90" s="2" t="inlineStr"/>
+          <t>You can submit only once. Check your Evidence board first.</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>paraphrase</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr"/>
@@ -3260,7 +3268,7 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>submit.keep_going</t>
+          <t>submit.choose</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -3270,7 +3278,7 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Keep investigating</t>
+          <t>— choose —</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr"/>
@@ -3284,17 +3292,17 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>result.correct</t>
+          <t>submit.both</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>Submission</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Case solved</t>
+          <t>Choose an answer for both questions.</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr"/>
@@ -3308,17 +3316,17 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>result.right_person_wrong_place</t>
+          <t>submit.submit</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>Submission</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Half right</t>
+          <t>Submit my solution</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr"/>
@@ -3332,17 +3340,17 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>result.wrong</t>
+          <t>submit.keep_going</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>Submission</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Not solved</t>
+          <t>Keep investigating</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr"/>
@@ -3356,7 +3364,7 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>result.you_named</t>
+          <t>result.correct</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -3366,7 +3374,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>You named {who} and “{where}”.</t>
+          <t>Case solved</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr"/>
@@ -3375,16 +3383,12 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F95" s="2" t="inlineStr">
-        <is>
-          <t>who where</t>
-        </is>
-      </c>
+      <c r="F95" s="2" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>result.one_more</t>
+          <t>result.right_person_wrong_place</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -3394,7 +3398,7 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>One more thing</t>
+          <t>Half right</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr"/>
@@ -3408,7 +3412,7 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>result.rank_prompt</t>
+          <t>result.wrong</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -3418,7 +3422,7 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Before the full story: how receptive was each witness? Rank them.</t>
+          <t>Not solved</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr"/>
@@ -3432,7 +3436,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>result.rank_button</t>
+          <t>result.you_named</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -3442,7 +3446,7 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Rank the witnesses</t>
+          <t>You named {who} and “{where}”.</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr"/>
@@ -3451,22 +3455,26 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F98" s="2" t="inlineStr"/>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>who where</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>ranking.title</t>
+          <t>result.one_more</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Ranking</t>
+          <t>Result</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Rank the witnesses by receptiveness</t>
+          <t>One more thing</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr"/>
@@ -3480,27 +3488,23 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>ranking.note</t>
+          <t>result.rank_prompt</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Ranking</t>
+          <t>Result</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Put the most receptive witness at the top and the least receptive at the bottom. Think about how they talked about the controversy, not whether they were helpful. You score {rank_exact} point for each witness in exactly the right place and {rank_near} for each one place off.</t>
-        </is>
-      </c>
-      <c r="D100" s="2" t="inlineStr">
-        <is>
-          <t>3.4</t>
-        </is>
-      </c>
+          <t>Before the full story: how receptive was each witness? Rank them.</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr"/>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>paraphrase</t>
+          <t>label</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr"/>
@@ -3508,17 +3512,17 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>ranking.submit</t>
+          <t>result.rank_button</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>Ranking</t>
+          <t>Result</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Submit ranking</t>
+          <t>Rank the witnesses</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr"/>
@@ -3532,17 +3536,17 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>ending.title</t>
+          <t>ranking.title</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Ending</t>
+          <t>Ranking</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Debrief</t>
+          <t>Rank the witnesses by receptiveness</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr"/>
@@ -3556,45 +3560,45 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>ending.verdict</t>
+          <t>ranking.note</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Ending</t>
+          <t>Ranking</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Verdict: **{verdict}**</t>
-        </is>
-      </c>
-      <c r="D103" s="2" t="inlineStr"/>
+          <t>Put the most receptive witness at the top and the least receptive at the bottom. Think about how they talked about the controversy, not whether they were helpful. You score {rank_exact} point for each witness in exactly the right place and {rank_near} for each one place off.</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>label</t>
-        </is>
-      </c>
-      <c r="F103" s="2" t="inlineStr">
-        <is>
-          <t>verdict</t>
-        </is>
-      </c>
+          <t>paraphrase</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>ending.verdict.correct</t>
+          <t>ranking.submit</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Ending</t>
+          <t>Ranking</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>solved</t>
+          <t>Submit ranking</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr"/>
@@ -3608,7 +3612,7 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>ending.verdict.right_person_wrong_place</t>
+          <t>ending.title</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -3618,7 +3622,7 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>half right</t>
+          <t>Debrief</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr"/>
@@ -3632,7 +3636,7 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>ending.verdict.wrong</t>
+          <t>ending.verdict</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -3642,7 +3646,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>not solved</t>
+          <t>Verdict: **{verdict}**</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr"/>
@@ -3651,12 +3655,16 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F106" s="2" t="inlineStr"/>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>ending.major</t>
+          <t>ending.verdict.correct</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -3666,7 +3674,7 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Major Clues earned: **{n} of {n_major}**</t>
+          <t>solved</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr"/>
@@ -3675,16 +3683,12 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F107" s="2" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
+      <c r="F107" s="2" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>ending.ranking</t>
+          <t>ending.verdict.right_person_wrong_place</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -3694,7 +3698,7 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Receptiveness ranking: **{score} of {n_witnesses}**</t>
+          <t>half right</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr"/>
@@ -3703,16 +3707,12 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F108" s="2" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
+      <c r="F108" s="2" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>ending.bonus</t>
+          <t>ending.verdict.wrong</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
@@ -3722,7 +3722,7 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>Follow-up bonus: **{points}**</t>
+          <t>not solved</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr"/>
@@ -3731,16 +3731,12 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F109" s="2" t="inlineStr">
-        <is>
-          <t>points</t>
-        </is>
-      </c>
+      <c r="F109" s="2" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>ending.used</t>
+          <t>ending.major</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -3750,7 +3746,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>Questions used: **{n} of {budget}**</t>
+          <t>Major Clues earned: **{n} of {n_major}**</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr"/>
@@ -3768,7 +3764,7 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>ending.table_title</t>
+          <t>ending.ranking</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
@@ -3778,7 +3774,7 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>Receptiveness, most to least</t>
+          <t>Receptiveness ranking: **{score} of {n_witnesses}**</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr"/>
@@ -3787,12 +3783,16 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F111" s="2" t="inlineStr"/>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>ending.col_rank</t>
+          <t>ending.bonus</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>Rank</t>
+          <t>Follow-up bonus: **{points}**</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr"/>
@@ -3811,12 +3811,16 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F112" s="2" t="inlineStr"/>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>points</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>ending.col_witness</t>
+          <t>ending.used</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
@@ -3826,7 +3830,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>Witness</t>
+          <t>Questions used: **{n} of {budget}**</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr"/>
@@ -3835,12 +3839,16 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F113" s="2" t="inlineStr"/>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>ending.col_yours</t>
+          <t>ending.table_title</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -3850,7 +3858,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>Your rank</t>
+          <t>Receptiveness, most to least</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr"/>
@@ -3864,7 +3872,7 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>ending.col_receptive</t>
+          <t>ending.col_rank</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
@@ -3874,7 +3882,7 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>Receptive answers</t>
+          <t>Rank</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr"/>
@@ -3888,7 +3896,7 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>ending.receptive_of</t>
+          <t>ending.col_witness</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -3898,7 +3906,7 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>{n} of {total}</t>
+          <t>Witness</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr"/>
@@ -3907,16 +3915,12 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F116" s="2" t="inlineStr">
-        <is>
-          <t>n total</t>
-        </is>
-      </c>
+      <c r="F116" s="2" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>ending.solution</t>
+          <t>ending.col_yours</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
@@ -3926,7 +3930,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>What really happened</t>
+          <t>Your rank</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr"/>
@@ -3940,7 +3944,7 @@
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>ending.full</t>
+          <t>ending.col_receptive</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
@@ -3950,7 +3954,7 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>The full ending</t>
+          <t>Receptive answers</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr"/>
@@ -3964,7 +3968,7 @@
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>ending.major_title</t>
+          <t>ending.receptive_of</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
@@ -3974,7 +3978,7 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>The Major Clues</t>
+          <t>{n} of {total}</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr"/>
@@ -3983,12 +3987,16 @@
           <t>label</t>
         </is>
       </c>
-      <c r="F119" s="2" t="inlineStr"/>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>n total</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>ending.herrings</t>
+          <t>ending.solution</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -3998,7 +4006,7 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>The red herrings, and how each one falls apart</t>
+          <t>What really happened</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr"/>
@@ -4012,7 +4020,7 @@
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>ending.again</t>
+          <t>ending.full</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
@@ -4022,7 +4030,7 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>Play again</t>
+          <t>The full ending</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr"/>
@@ -4032,6 +4040,78 @@
         </is>
       </c>
       <c r="F121" s="2" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>ending.major_title</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>Ending</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>The Major Clues</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr"/>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>ending.herrings</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>Ending</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>The red herrings, and how each one falls apart</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr"/>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>ending.again</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>Ending</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>Play again</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr"/>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>